<commit_message>
docs: REQ·API admin 연관화면 통합 정합 (v0.5)
admin 화면 통합(SUBS-02·PLAN-02·ORDER-01 제거)에 맞춰 연관화면 참조 갱신.
- API: 111/112→SUBS-01, 121/122→PLAN-01, 160/161→SHOP-01
- REQ: AD-003→SUBS-01, AD-006→PLAN-01, AD-010→SHOP-01
- 표지 v0.5, 변경이력 갱신. 검증: 3종 문서 dangling(SUBS-02/PLAN-02/ORDER-01/SHOP-02) 0.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ZIPBODA_API 및 인터페이스 정의서_v0.1.xlsx
+++ b/docs/ZIPBODA_API 및 인터페이스 정의서_v0.1.xlsx
@@ -869,11 +869,23 @@
       <c r="F6" s="21" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="50">
-      <c r="A7" s="21" t="n"/>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="24" t="n"/>
+      <c r="A7" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>admin 화면 통합 정합 — 연관화면 갱신(API-111/112→SUBS-01, 121/122→PLAN-01, 160/161→SHOP-01)</t>
+        </is>
+      </c>
       <c r="D7" s="21" t="n"/>
-      <c r="E7" s="30" t="n"/>
+      <c r="E7" s="30" t="n">
+        <v>46234</v>
+      </c>
       <c r="F7" s="21" t="n"/>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="50">
@@ -7674,7 +7686,7 @@
       </c>
       <c r="S55" s="47" t="inlineStr">
         <is>
-          <t>ZB-A-SUBS-02</t>
+          <t>ZB-A-SUBS-01</t>
         </is>
       </c>
       <c r="T55" s="47" t="inlineStr">
@@ -7779,7 +7791,7 @@
       </c>
       <c r="S56" s="47" t="inlineStr">
         <is>
-          <t>ZB-A-SUBS-02</t>
+          <t>ZB-A-SUBS-01</t>
         </is>
       </c>
       <c r="T56" s="47" t="inlineStr">
@@ -8209,7 +8221,7 @@
       </c>
       <c r="S60" s="47" t="inlineStr">
         <is>
-          <t>ZB-A-PLAN-02</t>
+          <t>ZB-A-PLAN-01</t>
         </is>
       </c>
       <c r="T60" s="47" t="inlineStr">
@@ -8319,7 +8331,7 @@
       </c>
       <c r="S61" s="47" t="inlineStr">
         <is>
-          <t>ZB-A-PLAN-02</t>
+          <t>ZB-A-PLAN-01</t>
         </is>
       </c>
       <c r="T61" s="47" t="inlineStr">
@@ -8657,7 +8669,7 @@
       </c>
       <c r="S64" s="47" t="inlineStr">
         <is>
-          <t>ZB-A-ORDER-01</t>
+          <t>ZB-A-SHOP-01</t>
         </is>
       </c>
       <c r="T64" s="47" t="inlineStr">
@@ -8770,7 +8782,7 @@
       </c>
       <c r="S65" s="47" t="inlineStr">
         <is>
-          <t>ZB-A-ORDER-01</t>
+          <t>ZB-A-SHOP-01</t>
         </is>
       </c>
       <c r="T65" s="47" t="inlineStr">

</xml_diff>